<commit_message>
addition of rate data
</commit_message>
<xml_diff>
--- a/utility data/Westminster/CoW Water Rates 2010-2025.xlsx
+++ b/utility data/Westminster/CoW Water Rates 2010-2025.xlsx
@@ -1,20 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://o365coloradoedu.sharepoint.com/sites/CEAE-HUB/Shared Documents/General/1 Projects/2025 Elasticity and Rate Structures CWCB/Jade/hub-gra-cwcb-rates/utility data/Westminster/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="42" documentId="13_ncr:1_{AB528C43-7210-4C1F-923F-CDC5F2149901}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D5808872-BD89-460C-8DA0-252788E8E13B}"/>
+  <xr:revisionPtr revIDLastSave="141" documentId="13_ncr:1_{AB528C43-7210-4C1F-923F-CDC5F2149901}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{268C1F2B-86FC-4C46-ADF9-1FFD8F07DEDF}"/>
   <bookViews>
-    <workbookView xWindow="25974" yWindow="-109" windowWidth="26301" windowHeight="14889" xr2:uid="{71E9F7F9-D1FB-4046-B409-886DDE225C90}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{71E9F7F9-D1FB-4046-B409-886DDE225C90}"/>
   </bookViews>
   <sheets>
-    <sheet name="SingleFamily" sheetId="1" r:id="rId1"/>
-    <sheet name="MultiFamily" sheetId="2" r:id="rId2"/>
+    <sheet name="Import-Prep" sheetId="3" r:id="rId1"/>
+    <sheet name="SingleFamily" sheetId="1" r:id="rId2"/>
+    <sheet name="MultiFamily" sheetId="2" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -36,8 +37,30 @@
 </workbook>
 </file>
 
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="1">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+</metadata>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="29">
   <si>
     <t>Block 1  1-6,000 gallons</t>
   </si>
@@ -94,6 +117,36 @@
   </si>
   <si>
     <t>Property management then distributes costs to tenants, in myriad different ways!</t>
+  </si>
+  <si>
+    <t>Residential, Single Family</t>
+  </si>
+  <si>
+    <t>Residential, Multi Family</t>
+  </si>
+  <si>
+    <t>cap_1</t>
+  </si>
+  <si>
+    <t>rate_1</t>
+  </si>
+  <si>
+    <t>cap_2</t>
+  </si>
+  <si>
+    <t>rate_2</t>
+  </si>
+  <si>
+    <t>cap_3</t>
+  </si>
+  <si>
+    <t>rate_3</t>
+  </si>
+  <si>
+    <t>Customer Category</t>
+  </si>
+  <si>
+    <t>Start Date</t>
   </si>
 </sst>
 </file>
@@ -138,7 +191,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -169,13 +222,65 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="5">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
       <diagonal/>
     </border>
   </borders>
@@ -184,7 +289,7 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="44" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="17" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -207,6 +312,24 @@
     <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Currency" xfId="1" builtinId="4"/>
@@ -542,378 +665,662 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A85E05AF-B576-4336-90E5-F96604FF0ED9}">
-  <dimension ref="A1:M27"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DFF596EA-6B15-4F7E-B590-F3A66927AA40}">
+  <sheetPr>
+    <tabColor theme="5"/>
+  </sheetPr>
+  <dimension ref="A1:H35"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="30.375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="22.7265625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="8.7265625" style="18"/>
+    <col min="3" max="3" width="7.6328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.7265625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="7.6328125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.7265625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="7.6328125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.7265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="B1">
-        <v>2010</v>
-      </c>
-      <c r="C1">
-        <v>2011</v>
-      </c>
-      <c r="D1">
-        <v>2012</v>
-      </c>
-      <c r="E1">
-        <v>2013</v>
-      </c>
-      <c r="F1">
-        <v>2014</v>
-      </c>
-      <c r="G1">
-        <v>2015</v>
-      </c>
-      <c r="H1">
-        <v>2016</v>
-      </c>
-      <c r="I1">
-        <v>2017</v>
-      </c>
-      <c r="J1">
-        <v>2018</v>
-      </c>
-      <c r="K1">
-        <v>2019</v>
-      </c>
-      <c r="L1">
-        <v>2020</v>
-      </c>
-      <c r="M1">
-        <v>2021</v>
-      </c>
-    </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" s="17" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="16" t="s">
+        <v>27</v>
+      </c>
+      <c r="B1" s="16" t="s">
+        <v>28</v>
+      </c>
+      <c r="C1" s="19" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1" s="20" t="s">
+        <v>22</v>
+      </c>
+      <c r="E1" s="19" t="s">
+        <v>23</v>
+      </c>
+      <c r="F1" s="20" t="s">
+        <v>24</v>
+      </c>
+      <c r="G1" s="19" t="s">
+        <v>25</v>
+      </c>
+      <c r="H1" s="20" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="1">
+        <v>19</v>
+      </c>
+      <c r="B2" s="18" cm="1">
+        <f t="array" ref="B2:B13">DATE(TRANSPOSE(SingleFamily!B1:M1),1,1)</f>
+        <v>40179</v>
+      </c>
+      <c r="C2" s="21">
+        <v>6000</v>
+      </c>
+      <c r="D2" s="22" cm="1">
+        <f t="array" ref="D2:D13">TRANSPOSE(SingleFamily!B2:M2)</f>
         <v>2.21</v>
       </c>
-      <c r="C2" s="1">
+      <c r="E2" s="21">
+        <v>20000</v>
+      </c>
+      <c r="F2" s="22" cm="1">
+        <f t="array" ref="F2:F13">TRANSPOSE(SingleFamily!B3:M3)</f>
+        <v>3.64</v>
+      </c>
+      <c r="G2" s="21"/>
+      <c r="H2" s="22" cm="1">
+        <f t="array" ref="H2:H13">TRANSPOSE(SingleFamily!B4:M4)</f>
+        <v>5.39</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="B3" s="18">
+        <v>40544</v>
+      </c>
+      <c r="C3" s="21">
+        <v>6000</v>
+      </c>
+      <c r="D3" s="22">
         <v>2.29</v>
       </c>
-      <c r="D2" s="1">
+      <c r="E3" s="21">
+        <v>20000</v>
+      </c>
+      <c r="F3" s="22">
+        <v>3.78</v>
+      </c>
+      <c r="G3" s="21"/>
+      <c r="H3" s="22">
+        <v>5.6</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="B4" s="18">
+        <v>40909</v>
+      </c>
+      <c r="C4" s="21">
+        <v>6000</v>
+      </c>
+      <c r="D4" s="22">
         <v>2.38</v>
       </c>
-      <c r="E2" s="1">
+      <c r="E4" s="21">
+        <v>20000</v>
+      </c>
+      <c r="F4" s="22">
+        <v>3.93</v>
+      </c>
+      <c r="G4" s="21"/>
+      <c r="H4" s="22">
+        <v>5.82</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="B5" s="18">
+        <v>41275</v>
+      </c>
+      <c r="C5" s="21">
+        <v>6000</v>
+      </c>
+      <c r="D5" s="22">
         <v>2.4700000000000002</v>
       </c>
-      <c r="F2" s="1">
+      <c r="E5" s="21">
+        <v>20000</v>
+      </c>
+      <c r="F5" s="22">
+        <v>4.08</v>
+      </c>
+      <c r="G5" s="21"/>
+      <c r="H5" s="22">
+        <v>6.05</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="B6" s="18">
+        <v>41640</v>
+      </c>
+      <c r="C6" s="21">
+        <v>6000</v>
+      </c>
+      <c r="D6" s="22">
         <v>2.56</v>
       </c>
-      <c r="G2" s="1">
+      <c r="E6" s="21">
+        <v>20000</v>
+      </c>
+      <c r="F6" s="22">
+        <v>4.24</v>
+      </c>
+      <c r="G6" s="21"/>
+      <c r="H6" s="22">
+        <v>6.29</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="B7" s="18">
+        <v>42005</v>
+      </c>
+      <c r="C7" s="21">
+        <v>6000</v>
+      </c>
+      <c r="D7" s="22">
         <v>2.66</v>
       </c>
-      <c r="H2" s="1">
+      <c r="E7" s="21">
+        <v>20000</v>
+      </c>
+      <c r="F7" s="22">
+        <v>4.4000000000000004</v>
+      </c>
+      <c r="G7" s="21"/>
+      <c r="H7" s="22">
+        <v>6.54</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="B8" s="18">
+        <v>42370</v>
+      </c>
+      <c r="C8" s="21">
+        <v>6000</v>
+      </c>
+      <c r="D8" s="22">
         <v>2.76</v>
       </c>
-      <c r="I2" s="1">
+      <c r="E8" s="21">
+        <v>20000</v>
+      </c>
+      <c r="F8" s="22">
+        <v>4.57</v>
+      </c>
+      <c r="G8" s="21"/>
+      <c r="H8" s="22">
+        <v>6.8016000000000005</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="B9" s="18">
+        <v>42736</v>
+      </c>
+      <c r="C9" s="21">
+        <v>6000</v>
+      </c>
+      <c r="D9" s="22">
         <v>2.98</v>
       </c>
-      <c r="J2" s="1">
+      <c r="E9" s="21">
+        <v>20000</v>
+      </c>
+      <c r="F9" s="22">
+        <v>4.93</v>
+      </c>
+      <c r="G9" s="21"/>
+      <c r="H9" s="22">
+        <v>7.34</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="B10" s="18">
+        <v>43101</v>
+      </c>
+      <c r="C10" s="21">
+        <v>6000</v>
+      </c>
+      <c r="D10" s="22">
         <v>3.22</v>
       </c>
-      <c r="K2" s="1">
+      <c r="E10" s="21">
+        <v>20000</v>
+      </c>
+      <c r="F10" s="22">
+        <v>5.32</v>
+      </c>
+      <c r="G10" s="21"/>
+      <c r="H10" s="22">
+        <v>7.93</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="B11" s="18">
+        <v>43466</v>
+      </c>
+      <c r="C11" s="21">
+        <v>6000</v>
+      </c>
+      <c r="D11" s="22">
         <v>3.57</v>
       </c>
-      <c r="L2" s="1">
+      <c r="E11" s="21">
+        <v>20000</v>
+      </c>
+      <c r="F11" s="22">
+        <v>7.35</v>
+      </c>
+      <c r="G11" s="21"/>
+      <c r="H11" s="22">
+        <v>11.62</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="B12" s="18">
+        <v>43831</v>
+      </c>
+      <c r="C12" s="21">
+        <v>6000</v>
+      </c>
+      <c r="D12" s="22">
         <v>3.96</v>
       </c>
-      <c r="M2" s="1">
+      <c r="E12" s="21">
+        <v>20000</v>
+      </c>
+      <c r="F12" s="22">
+        <v>8.15</v>
+      </c>
+      <c r="G12" s="21"/>
+      <c r="H12" s="22">
+        <v>12.88</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="B13" s="18">
+        <v>44197</v>
+      </c>
+      <c r="C13" s="21">
+        <v>6000</v>
+      </c>
+      <c r="D13" s="22">
         <v>3.96</v>
       </c>
-    </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>1</v>
-      </c>
-      <c r="B3" s="1">
-        <v>3.64</v>
-      </c>
-      <c r="C3" s="1">
-        <v>3.78</v>
-      </c>
-      <c r="D3" s="1">
-        <v>3.93</v>
-      </c>
-      <c r="E3" s="1">
-        <v>4.08</v>
-      </c>
-      <c r="F3" s="1">
-        <v>4.24</v>
-      </c>
-      <c r="G3" s="1">
-        <v>4.4000000000000004</v>
-      </c>
-      <c r="H3" s="1">
-        <v>4.57</v>
-      </c>
-      <c r="I3" s="1">
-        <v>4.93</v>
-      </c>
-      <c r="J3" s="1">
-        <v>5.32</v>
-      </c>
-      <c r="K3" s="6">
-        <v>7.35</v>
-      </c>
-      <c r="L3" s="1">
+      <c r="E13" s="21">
+        <v>20000</v>
+      </c>
+      <c r="F13" s="22">
         <v>8.15</v>
       </c>
-      <c r="M3" s="4">
+      <c r="G13" s="21"/>
+      <c r="H13" s="22">
+        <v>12.88</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="B14" s="18">
+        <f>SingleFamily!B6</f>
+        <v>44562</v>
+      </c>
+      <c r="C14" s="21">
+        <v>6000</v>
+      </c>
+      <c r="D14" s="22">
+        <f>SingleFamily!B7</f>
+        <v>3.96</v>
+      </c>
+      <c r="E14" s="21">
+        <v>20000</v>
+      </c>
+      <c r="F14" s="22">
+        <f>SingleFamily!B8</f>
         <v>8.15</v>
       </c>
-    </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>2</v>
-      </c>
-      <c r="B4" s="1">
-        <v>5.39</v>
-      </c>
-      <c r="C4" s="1">
-        <v>5.6</v>
-      </c>
-      <c r="D4" s="1">
-        <v>5.82</v>
-      </c>
-      <c r="E4" s="1">
-        <v>6.05</v>
-      </c>
-      <c r="F4" s="1">
-        <v>6.29</v>
-      </c>
-      <c r="G4" s="1">
-        <v>6.54</v>
-      </c>
-      <c r="H4" s="1">
-        <v>6.8016000000000005</v>
-      </c>
-      <c r="I4" s="1">
-        <v>7.34</v>
-      </c>
-      <c r="J4" s="1">
-        <v>7.93</v>
-      </c>
-      <c r="K4" s="6">
-        <v>11.62</v>
-      </c>
-      <c r="L4" s="1">
+      <c r="G14" s="21"/>
+      <c r="H14" s="22">
+        <f>SingleFamily!B9</f>
         <v>12.88</v>
       </c>
-      <c r="M4" s="4">
-        <v>12.88</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="B6" s="2">
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="B15" s="18">
+        <f>SingleFamily!B11</f>
+        <v>44621</v>
+      </c>
+      <c r="C15" s="21">
+        <v>6000</v>
+      </c>
+      <c r="D15" s="22">
+        <f>SingleFamily!B12</f>
+        <v>3.96</v>
+      </c>
+      <c r="E15" s="21">
+        <v>20000</v>
+      </c>
+      <c r="F15" s="22">
+        <f>SingleFamily!B13</f>
+        <v>8.15</v>
+      </c>
+      <c r="G15" s="21"/>
+      <c r="H15" s="22">
+        <f>SingleFamily!B14</f>
+        <v>8.15</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="B16" s="18">
+        <f>SingleFamily!B16</f>
+        <v>44713</v>
+      </c>
+      <c r="C16" s="21">
+        <v>8000</v>
+      </c>
+      <c r="D16" s="22">
+        <f>SingleFamily!B17</f>
+        <v>3.57</v>
+      </c>
+      <c r="E16" s="21">
+        <v>40000</v>
+      </c>
+      <c r="F16" s="22">
+        <f>SingleFamily!B18</f>
+        <v>6.52</v>
+      </c>
+      <c r="G16" s="21"/>
+      <c r="H16" s="22">
+        <f>SingleFamily!B19</f>
+        <v>8.15</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="B17" s="18" cm="1">
+        <f t="array" ref="B17:B19">DATE(TRANSPOSE(SingleFamily!B21:D21),1,1)</f>
+        <v>44927</v>
+      </c>
+      <c r="C17" s="21">
+        <v>8000</v>
+      </c>
+      <c r="D17" s="22" cm="1">
+        <f t="array" ref="D17:D19">TRANSPOSE(SingleFamily!B22:D22)</f>
+        <v>3.7128000000000001</v>
+      </c>
+      <c r="E17" s="21">
+        <v>40000</v>
+      </c>
+      <c r="F17" s="22" cm="1">
+        <f t="array" ref="F17:F19">TRANSPOSE(SingleFamily!B23:D23)</f>
+        <v>6.7808000000000002</v>
+      </c>
+      <c r="G17" s="21"/>
+      <c r="H17" s="22" cm="1">
+        <f t="array" ref="H17:H19">TRANSPOSE(SingleFamily!B24:D24)</f>
+        <v>8.4760000000000009</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="B18" s="18">
+        <v>45292</v>
+      </c>
+      <c r="C18" s="21">
+        <v>8000</v>
+      </c>
+      <c r="D18" s="22">
+        <v>3.8798759999999999</v>
+      </c>
+      <c r="E18" s="21">
+        <v>40000</v>
+      </c>
+      <c r="F18" s="22">
+        <v>7.0859359999999993</v>
+      </c>
+      <c r="G18" s="21"/>
+      <c r="H18" s="22">
+        <v>8.8574200000000012</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="B19" s="18">
+        <v>45658</v>
+      </c>
+      <c r="C19" s="21">
+        <v>8000</v>
+      </c>
+      <c r="D19" s="22">
+        <v>4.0350710400000001</v>
+      </c>
+      <c r="E19" s="21">
+        <v>40000</v>
+      </c>
+      <c r="F19" s="22">
+        <v>7.3693734400000004</v>
+      </c>
+      <c r="G19" s="21"/>
+      <c r="H19" s="22">
+        <v>9.2117167999999996</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
+        <v>20</v>
+      </c>
+      <c r="B20" s="18" cm="1">
+        <f t="array" ref="B20:B35">DATE(TRANSPOSE(MultiFamily!B1:Q1),1,1)</f>
+        <v>40179</v>
+      </c>
+      <c r="C20" s="21"/>
+      <c r="D20" s="22" cm="1">
+        <f t="array" ref="D20:D35">TRANSPOSE(MultiFamily!B2:Q2)</f>
+        <v>4.5199999999999996</v>
+      </c>
+      <c r="E20" s="21"/>
+      <c r="F20" s="22"/>
+      <c r="G20" s="21"/>
+      <c r="H20" s="22"/>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="B21" s="18">
+        <v>40544</v>
+      </c>
+      <c r="C21" s="21"/>
+      <c r="D21" s="22">
+        <v>4.7</v>
+      </c>
+      <c r="E21" s="21"/>
+      <c r="F21" s="22"/>
+      <c r="G21" s="21"/>
+      <c r="H21" s="22"/>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="B22" s="18">
+        <v>40909</v>
+      </c>
+      <c r="C22" s="21"/>
+      <c r="D22" s="22">
+        <v>4.88</v>
+      </c>
+      <c r="E22" s="21"/>
+      <c r="F22" s="22"/>
+      <c r="G22" s="21"/>
+      <c r="H22" s="22"/>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="B23" s="18">
+        <v>41275</v>
+      </c>
+      <c r="C23" s="21"/>
+      <c r="D23" s="22">
+        <v>5.07</v>
+      </c>
+      <c r="E23" s="21"/>
+      <c r="F23" s="22"/>
+      <c r="G23" s="21"/>
+      <c r="H23" s="22"/>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="B24" s="18">
+        <v>41640</v>
+      </c>
+      <c r="C24" s="21"/>
+      <c r="D24" s="22">
+        <v>5.27</v>
+      </c>
+      <c r="E24" s="21"/>
+      <c r="F24" s="22"/>
+      <c r="G24" s="21"/>
+      <c r="H24" s="22"/>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="B25" s="18">
+        <v>42005</v>
+      </c>
+      <c r="C25" s="21"/>
+      <c r="D25" s="22">
+        <v>5.48</v>
+      </c>
+      <c r="E25" s="21"/>
+      <c r="F25" s="22"/>
+      <c r="G25" s="21"/>
+      <c r="H25" s="22"/>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="B26" s="18">
+        <v>42370</v>
+      </c>
+      <c r="C26" s="21"/>
+      <c r="D26" s="22">
+        <v>5.69</v>
+      </c>
+      <c r="E26" s="21"/>
+      <c r="F26" s="22"/>
+      <c r="G26" s="21"/>
+      <c r="H26" s="22"/>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="B27" s="18">
+        <v>42736</v>
+      </c>
+      <c r="C27" s="21"/>
+      <c r="D27" s="22">
+        <v>6.14</v>
+      </c>
+      <c r="E27" s="21"/>
+      <c r="F27" s="22"/>
+      <c r="G27" s="21"/>
+      <c r="H27" s="22"/>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="B28" s="18">
+        <v>43101</v>
+      </c>
+      <c r="C28" s="21"/>
+      <c r="D28" s="22">
+        <v>6.63</v>
+      </c>
+      <c r="E28" s="21"/>
+      <c r="F28" s="22"/>
+      <c r="G28" s="21"/>
+      <c r="H28" s="22"/>
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="B29" s="18">
+        <v>43466</v>
+      </c>
+      <c r="C29" s="21"/>
+      <c r="D29" s="22">
+        <v>7.11</v>
+      </c>
+      <c r="E29" s="21"/>
+      <c r="F29" s="22"/>
+      <c r="G29" s="21"/>
+      <c r="H29" s="22"/>
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="B30" s="18">
+        <v>43831</v>
+      </c>
+      <c r="C30" s="21"/>
+      <c r="D30" s="22">
+        <v>7.55</v>
+      </c>
+      <c r="E30" s="21"/>
+      <c r="F30" s="22"/>
+      <c r="G30" s="21"/>
+      <c r="H30" s="22"/>
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="B31" s="18">
+        <v>44197</v>
+      </c>
+      <c r="C31" s="21"/>
+      <c r="D31" s="22">
+        <v>7.55</v>
+      </c>
+      <c r="E31" s="21"/>
+      <c r="F31" s="22"/>
+      <c r="G31" s="21"/>
+      <c r="H31" s="22"/>
+    </row>
+    <row r="32" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="B32" s="18">
         <v>44562</v>
       </c>
-    </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>0</v>
-      </c>
-      <c r="B7" s="1">
-        <v>3.96</v>
-      </c>
-      <c r="D7" s="5" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>1</v>
-      </c>
-      <c r="B8" s="1">
-        <v>8.15</v>
-      </c>
-      <c r="D8" s="7">
-        <v>2019</v>
-      </c>
-      <c r="E8" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>2</v>
-      </c>
-      <c r="B9" s="1">
-        <v>12.88</v>
-      </c>
-      <c r="D9" s="8">
-        <v>2021</v>
-      </c>
-      <c r="E9" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="D10" s="10">
-        <v>44621</v>
-      </c>
-      <c r="E10" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="B11" s="2">
-        <v>44621</v>
-      </c>
-      <c r="D11" s="11">
-        <v>44713</v>
-      </c>
-      <c r="E11" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>0</v>
-      </c>
-      <c r="B12" s="1">
-        <v>3.96</v>
-      </c>
-    </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>1</v>
-      </c>
-      <c r="B13" s="1">
-        <v>8.15</v>
-      </c>
-    </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>2</v>
-      </c>
-      <c r="B14" s="9">
-        <v>8.15</v>
-      </c>
-      <c r="G14" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="G15" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="B16" s="2">
-        <v>44713</v>
-      </c>
-      <c r="G16" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A17" s="12" t="s">
-        <v>8</v>
-      </c>
-      <c r="B17" s="13">
-        <v>3.57</v>
-      </c>
-      <c r="G17" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A18" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="B18" s="13">
-        <v>6.52</v>
-      </c>
-    </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A19" s="12" t="s">
-        <v>10</v>
-      </c>
-      <c r="B19" s="13">
-        <v>8.15</v>
-      </c>
-    </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B21">
-        <v>2023</v>
-      </c>
-      <c r="C21">
-        <v>2024</v>
-      </c>
-      <c r="D21">
-        <v>2025</v>
-      </c>
-    </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A22" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="B22" s="1">
-        <f>3.57*1.04</f>
-        <v>3.7128000000000001</v>
-      </c>
-      <c r="C22" s="1">
-        <f>3.7128*1.045</f>
-        <v>3.8798759999999999</v>
-      </c>
-      <c r="D22" s="1">
-        <f>3.879876*1.04</f>
-        <v>4.0350710400000001</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A23" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="B23" s="1">
-        <f>6.52*1.04</f>
-        <v>6.7808000000000002</v>
-      </c>
-      <c r="C23" s="1">
-        <f>6.7808*1.045</f>
-        <v>7.0859359999999993</v>
-      </c>
-      <c r="D23" s="1">
-        <f>7.085936*1.04</f>
-        <v>7.3693734400000004</v>
-      </c>
-    </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A24" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="B24" s="1">
-        <f>8.15*1.04</f>
-        <v>8.4760000000000009</v>
-      </c>
-      <c r="C24" s="1">
-        <f>8.476*1.045</f>
-        <v>8.8574200000000012</v>
-      </c>
-      <c r="D24" s="1">
-        <f>8.85742*1.04</f>
-        <v>9.2117167999999996</v>
-      </c>
-    </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B25" s="1"/>
-      <c r="C25" s="1"/>
-      <c r="D25" s="1"/>
-      <c r="F25" s="1"/>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="F26" s="1"/>
-    </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="F27" s="1"/>
+      <c r="C32" s="21"/>
+      <c r="D32" s="22">
+        <v>7.55</v>
+      </c>
+      <c r="E32" s="21"/>
+      <c r="F32" s="22"/>
+      <c r="G32" s="21"/>
+      <c r="H32" s="22"/>
+    </row>
+    <row r="33" spans="2:8" x14ac:dyDescent="0.35">
+      <c r="B33" s="18">
+        <v>44927</v>
+      </c>
+      <c r="C33" s="21"/>
+      <c r="D33" s="22">
+        <v>7.85</v>
+      </c>
+      <c r="E33" s="21"/>
+      <c r="F33" s="22"/>
+      <c r="G33" s="21"/>
+      <c r="H33" s="22"/>
+    </row>
+    <row r="34" spans="2:8" x14ac:dyDescent="0.35">
+      <c r="B34" s="18">
+        <v>45292</v>
+      </c>
+      <c r="C34" s="21"/>
+      <c r="D34" s="22">
+        <v>8.2100000000000009</v>
+      </c>
+      <c r="E34" s="21"/>
+      <c r="F34" s="22"/>
+      <c r="G34" s="21"/>
+      <c r="H34" s="22"/>
+    </row>
+    <row r="35" spans="2:8" x14ac:dyDescent="0.35">
+      <c r="B35" s="18">
+        <v>45658</v>
+      </c>
+      <c r="C35" s="23"/>
+      <c r="D35" s="24">
+        <v>8.5299999999999994</v>
+      </c>
+      <c r="E35" s="23"/>
+      <c r="F35" s="24"/>
+      <c r="G35" s="23"/>
+      <c r="H35" s="24"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -921,14 +1328,393 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A85E05AF-B576-4336-90E5-F96604FF0ED9}">
+  <dimension ref="A1:M27"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="30.36328125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.08984375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="B1">
+        <v>2010</v>
+      </c>
+      <c r="C1">
+        <v>2011</v>
+      </c>
+      <c r="D1">
+        <v>2012</v>
+      </c>
+      <c r="E1">
+        <v>2013</v>
+      </c>
+      <c r="F1">
+        <v>2014</v>
+      </c>
+      <c r="G1">
+        <v>2015</v>
+      </c>
+      <c r="H1">
+        <v>2016</v>
+      </c>
+      <c r="I1">
+        <v>2017</v>
+      </c>
+      <c r="J1">
+        <v>2018</v>
+      </c>
+      <c r="K1">
+        <v>2019</v>
+      </c>
+      <c r="L1">
+        <v>2020</v>
+      </c>
+      <c r="M1">
+        <v>2021</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="1">
+        <v>2.21</v>
+      </c>
+      <c r="C2" s="1">
+        <v>2.29</v>
+      </c>
+      <c r="D2" s="1">
+        <v>2.38</v>
+      </c>
+      <c r="E2" s="1">
+        <v>2.4700000000000002</v>
+      </c>
+      <c r="F2" s="1">
+        <v>2.56</v>
+      </c>
+      <c r="G2" s="1">
+        <v>2.66</v>
+      </c>
+      <c r="H2" s="1">
+        <v>2.76</v>
+      </c>
+      <c r="I2" s="1">
+        <v>2.98</v>
+      </c>
+      <c r="J2" s="1">
+        <v>3.22</v>
+      </c>
+      <c r="K2" s="1">
+        <v>3.57</v>
+      </c>
+      <c r="L2" s="1">
+        <v>3.96</v>
+      </c>
+      <c r="M2" s="1">
+        <v>3.96</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" s="1">
+        <v>3.64</v>
+      </c>
+      <c r="C3" s="1">
+        <v>3.78</v>
+      </c>
+      <c r="D3" s="1">
+        <v>3.93</v>
+      </c>
+      <c r="E3" s="1">
+        <v>4.08</v>
+      </c>
+      <c r="F3" s="1">
+        <v>4.24</v>
+      </c>
+      <c r="G3" s="1">
+        <v>4.4000000000000004</v>
+      </c>
+      <c r="H3" s="1">
+        <v>4.57</v>
+      </c>
+      <c r="I3" s="1">
+        <v>4.93</v>
+      </c>
+      <c r="J3" s="1">
+        <v>5.32</v>
+      </c>
+      <c r="K3" s="6">
+        <v>7.35</v>
+      </c>
+      <c r="L3" s="1">
+        <v>8.15</v>
+      </c>
+      <c r="M3" s="4">
+        <v>8.15</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4" s="1">
+        <v>5.39</v>
+      </c>
+      <c r="C4" s="1">
+        <v>5.6</v>
+      </c>
+      <c r="D4" s="1">
+        <v>5.82</v>
+      </c>
+      <c r="E4" s="1">
+        <v>6.05</v>
+      </c>
+      <c r="F4" s="1">
+        <v>6.29</v>
+      </c>
+      <c r="G4" s="1">
+        <v>6.54</v>
+      </c>
+      <c r="H4" s="1">
+        <v>6.8016000000000005</v>
+      </c>
+      <c r="I4" s="1">
+        <v>7.34</v>
+      </c>
+      <c r="J4" s="1">
+        <v>7.93</v>
+      </c>
+      <c r="K4" s="6">
+        <v>11.62</v>
+      </c>
+      <c r="L4" s="1">
+        <v>12.88</v>
+      </c>
+      <c r="M4" s="4">
+        <v>12.88</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="B6" s="2">
+        <v>44562</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>0</v>
+      </c>
+      <c r="B7" s="1">
+        <v>3.96</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>1</v>
+      </c>
+      <c r="B8" s="1">
+        <v>8.15</v>
+      </c>
+      <c r="D8" s="7">
+        <v>2019</v>
+      </c>
+      <c r="E8" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>2</v>
+      </c>
+      <c r="B9" s="1">
+        <v>12.88</v>
+      </c>
+      <c r="D9" s="8">
+        <v>2021</v>
+      </c>
+      <c r="E9" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="D10" s="10">
+        <v>44621</v>
+      </c>
+      <c r="E10" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="B11" s="2">
+        <v>44621</v>
+      </c>
+      <c r="D11" s="11">
+        <v>44713</v>
+      </c>
+      <c r="E11" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>0</v>
+      </c>
+      <c r="B12" s="1">
+        <v>3.96</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>1</v>
+      </c>
+      <c r="B13" s="1">
+        <v>8.15</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
+        <v>2</v>
+      </c>
+      <c r="B14" s="9">
+        <v>8.15</v>
+      </c>
+      <c r="G14" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="G15" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="16" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="B16" s="2">
+        <v>44713</v>
+      </c>
+      <c r="G16" s="25" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A17" s="12" t="s">
+        <v>8</v>
+      </c>
+      <c r="B17" s="13">
+        <v>3.57</v>
+      </c>
+      <c r="G17" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A18" s="12" t="s">
+        <v>9</v>
+      </c>
+      <c r="B18" s="13">
+        <v>6.52</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A19" s="12" t="s">
+        <v>10</v>
+      </c>
+      <c r="B19" s="13">
+        <v>8.15</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="B21">
+        <v>2023</v>
+      </c>
+      <c r="C21">
+        <v>2024</v>
+      </c>
+      <c r="D21">
+        <v>2025</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A22" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B22" s="1">
+        <f>3.57*1.04</f>
+        <v>3.7128000000000001</v>
+      </c>
+      <c r="C22" s="1">
+        <f>3.7128*1.045</f>
+        <v>3.8798759999999999</v>
+      </c>
+      <c r="D22" s="1">
+        <f>3.879876*1.04</f>
+        <v>4.0350710400000001</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A23" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B23" s="1">
+        <f>6.52*1.04</f>
+        <v>6.7808000000000002</v>
+      </c>
+      <c r="C23" s="1">
+        <f>6.7808*1.045</f>
+        <v>7.0859359999999993</v>
+      </c>
+      <c r="D23" s="1">
+        <f>7.085936*1.04</f>
+        <v>7.3693734400000004</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A24" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B24" s="1">
+        <f>8.15*1.04</f>
+        <v>8.4760000000000009</v>
+      </c>
+      <c r="C24" s="1">
+        <f>8.476*1.045</f>
+        <v>8.8574200000000012</v>
+      </c>
+      <c r="D24" s="1">
+        <f>8.85742*1.04</f>
+        <v>9.2117167999999996</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="B25" s="1"/>
+      <c r="C25" s="1"/>
+      <c r="D25" s="1"/>
+      <c r="F25" s="1"/>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="F26" s="1"/>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="F27" s="1"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AED9540D-AAD1-4884-A298-B1A224CFF7A1}">
   <dimension ref="A1:Q6"/>
-  <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="27.75" customWidth="1"/>
+    <col min="1" max="1" width="27.7265625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:17" x14ac:dyDescent="0.35">
       <c r="B1">
         <v>2010</v>
       </c>
@@ -978,7 +1764,7 @@
         <v>2025</v>
       </c>
     </row>
-    <row r="2" spans="1:17" ht="42.8" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:17" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A2" s="14" t="s">
         <v>15</v>
       </c>
@@ -1031,17 +1817,17 @@
         <v>8.5299999999999994</v>
       </c>
     </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:17" x14ac:dyDescent="0.35">
       <c r="B4" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:17" x14ac:dyDescent="0.35">
       <c r="B5" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:17" x14ac:dyDescent="0.35">
       <c r="B6" t="s">
         <v>18</v>
       </c>
@@ -1052,6 +1838,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <TaxCatchAll xmlns="68738bc9-97b6-4aea-9722-c8130ccafb9b" xsi:nil="true"/>
@@ -1062,9 +1857,9 @@
 </p:properties>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010095E869ECB1E35142B7986647353A6071" ma:contentTypeVersion="16" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="bd59a79325bdce54e5e21e2629eabd4a">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="43e0f7cf-9242-4a2b-99ce-72db65c8030e" xmlns:ns3="68738bc9-97b6-4aea-9722-c8130ccafb9b" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="fce0723309a65e62c1e02d4838c24021" ns2:_="" ns3:_="">
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010095E869ECB1E35142B7986647353A6071" ma:contentTypeVersion="16" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="cbcba10418e375a4867da0970ef9eaff">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="43e0f7cf-9242-4a2b-99ce-72db65c8030e" xmlns:ns3="68738bc9-97b6-4aea-9722-c8130ccafb9b" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="d5f766f5a5c1c31e68546498d07283b9" ns2:_="" ns3:_="">
     <xsd:import namespace="43e0f7cf-9242-4a2b-99ce-72db65c8030e"/>
     <xsd:import namespace="68738bc9-97b6-4aea-9722-c8130ccafb9b"/>
     <xsd:element name="properties">
@@ -1303,16 +2098,15 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{42436099-1549-4141-BB42-1C055EF25ABE}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FF3F04D6-3455-4156-B2D9-26364E1CC390}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
@@ -1329,8 +2123,8 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{528CB3C6-855B-4D14-8D12-C15DB5A335E9}">
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{07BDBBFC-15D5-4CBC-B752-E8465775A9EF}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
@@ -1346,12 +2140,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{42436099-1549-4141-BB42-1C055EF25ABE}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>